<commit_message>
visualização de empréstimos ativos
</commit_message>
<xml_diff>
--- a/Caixinha 2026.xlsx
+++ b/Caixinha 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/368431def48b862b/Banco Gênio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="315" documentId="8_{8553A8CE-1C28-4DA3-90E5-ABB7540879BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C570641-88BA-4B90-A8ED-D408345A9F08}"/>
+  <xr:revisionPtr revIDLastSave="517" documentId="8_{8553A8CE-1C28-4DA3-90E5-ABB7540879BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{128DDA40-EA49-4735-A840-D8609E947D56}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{7BE32042-2CEA-4C59-BC4F-84862DE40344}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="5" xr2:uid="{7BE32042-2CEA-4C59-BC4F-84862DE40344}"/>
   </bookViews>
   <sheets>
     <sheet name="Participantes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="99">
   <si>
     <t>Nome</t>
   </si>
@@ -308,6 +308,42 @@
   </si>
   <si>
     <t>Não</t>
+  </si>
+  <si>
+    <t>Fevereiro</t>
+  </si>
+  <si>
+    <t>f631A</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>Saída</t>
+  </si>
+  <si>
+    <t>f641A</t>
+  </si>
+  <si>
+    <t>f651E</t>
+  </si>
+  <si>
+    <t>Adriana dos reis mota progenio</t>
+  </si>
+  <si>
+    <t>92640591215</t>
+  </si>
+  <si>
+    <t>J632A</t>
+  </si>
+  <si>
+    <t>m632E</t>
+  </si>
+  <si>
+    <t>Março</t>
+  </si>
+  <si>
+    <t>m631E</t>
   </si>
 </sst>
 </file>
@@ -459,6 +495,9 @@
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <left style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -498,9 +537,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -532,33 +568,33 @@
       <sheetName val="Tesouro direto"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1">
         <row r="14">
           <cell r="C14">
-            <v>21992.66105212655</v>
+            <v>21320.658425285445</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F490DB45-F4EA-40A7-A145-87F7EAC00B0B}" name="participantes" displayName="participantes" ref="A1:K3" totalsRowShown="0">
-  <autoFilter ref="A1:K3" xr:uid="{F490DB45-F4EA-40A7-A145-87F7EAC00B0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F490DB45-F4EA-40A7-A145-87F7EAC00B0B}" name="participantes" displayName="participantes" ref="A1:K4" totalsRowShown="0">
+  <autoFilter ref="A1:K4" xr:uid="{F490DB45-F4EA-40A7-A145-87F7EAC00B0B}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{998788C2-B6CB-4302-92E4-6D559237E9BD}" name="ID"/>
     <tableColumn id="2" xr3:uid="{9B11F552-3C83-47B9-B8E0-A21D3921B26F}" name="Nome"/>
-    <tableColumn id="3" xr3:uid="{6608BBC3-BA8D-4AC2-91DD-FD0A08445FE0}" name="CPF" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{6608BBC3-BA8D-4AC2-91DD-FD0A08445FE0}" name="CPF" dataDxfId="11"/>
     <tableColumn id="4" xr3:uid="{C06694F4-69AD-48F5-BCD6-C8242BF75D6B}" name="Endereço"/>
     <tableColumn id="5" xr3:uid="{07F7C9E3-EF6C-490C-8758-A8C1F1486002}" name="E-mail" dataCellStyle="Hiperlink"/>
     <tableColumn id="6" xr3:uid="{3739A20B-13B5-4FCF-A7A6-6B93A07AF3D4}" name="Telefone"/>
@@ -579,7 +615,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{700E6658-495C-4A79-A0A6-D6C1461C4A22}" name="Tabela5" displayName="Tabela5" ref="A1:C5" totalsRowShown="0" headerRowDxfId="12" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{700E6658-495C-4A79-A0A6-D6C1461C4A22}" name="Tabela5" displayName="Tabela5" ref="A1:C5" totalsRowShown="0" headerRowDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A1:C5" xr:uid="{700E6658-495C-4A79-A0A6-D6C1461C4A22}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{70364159-8838-4F57-959F-06AED0DFD52E}" name="Descrição"/>
@@ -591,8 +627,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2F57D50C-8D9F-4AB1-9907-E1255F5EAF6E}" name="Investimentos" displayName="Investimentos" ref="A1:K4" totalsRowShown="0">
-  <autoFilter ref="A1:K4" xr:uid="{2F57D50C-8D9F-4AB1-9907-E1255F5EAF6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2F57D50C-8D9F-4AB1-9907-E1255F5EAF6E}" name="Investimentos" displayName="Investimentos" ref="A1:K9" totalsRowShown="0">
+  <autoFilter ref="A1:K9" xr:uid="{2F57D50C-8D9F-4AB1-9907-E1255F5EAF6E}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{2094E236-758F-462B-A88B-0B1F3B8771B0}" name="Código"/>
     <tableColumn id="2" xr3:uid="{ED20D07D-11CA-470E-BD3C-3DB3914D8621}" name="OBS"/>
@@ -623,8 +659,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AFB1159D-14A2-49BA-85BE-A44737C6E3CB}" name="Tabela7" displayName="Tabela7" ref="A1:N3" totalsRowShown="0">
-  <autoFilter ref="A1:N3" xr:uid="{AFB1159D-14A2-49BA-85BE-A44737C6E3CB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{AFB1159D-14A2-49BA-85BE-A44737C6E3CB}" name="Tabela7" displayName="Tabela7" ref="A1:N4" totalsRowShown="0">
+  <autoFilter ref="A1:N4" xr:uid="{AFB1159D-14A2-49BA-85BE-A44737C6E3CB}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{C60B0CF5-8050-484C-89F4-017E3D8960E2}" name="ID"/>
     <tableColumn id="2" xr3:uid="{D66E2CD6-7E46-4A3B-BC49-24F30FFE5689}" name="ID Participante"/>
@@ -654,8 +690,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2C891125-C088-4223-AFED-A62E56738F56}" name="Emprestimos" displayName="Emprestimos" ref="A1:K2" totalsRowShown="0">
-  <autoFilter ref="A1:K2" xr:uid="{2C891125-C088-4223-AFED-A62E56738F56}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2C891125-C088-4223-AFED-A62E56738F56}" name="Emprestimos" displayName="Emprestimos" ref="A1:K4" totalsRowShown="0">
+  <autoFilter ref="A1:K4" xr:uid="{2C891125-C088-4223-AFED-A62E56738F56}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{1F38CEF8-8A61-4F0C-AFBE-E36D13DF7303}" name="ID"/>
     <tableColumn id="2" xr3:uid="{8D6D6EBE-208E-432B-BF48-5E2E229A661A}" name="id_participante"/>
@@ -680,8 +716,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CBB5763A-BBCD-4FF9-8A7F-7C2DE477406C}" name="Parcelas" displayName="Parcelas" ref="A1:G3" totalsRowShown="0">
-  <autoFilter ref="A1:G3" xr:uid="{CBB5763A-BBCD-4FF9-8A7F-7C2DE477406C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{CBB5763A-BBCD-4FF9-8A7F-7C2DE477406C}" name="Parcelas" displayName="Parcelas" ref="A1:G6" totalsRowShown="0">
+  <autoFilter ref="A1:G6" xr:uid="{CBB5763A-BBCD-4FF9-8A7F-7C2DE477406C}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B5BD6FB6-85AD-4333-BD59-D2D94F342BF2}" name="ID"/>
     <tableColumn id="2" xr3:uid="{B2220499-6820-4172-9C93-262080414420}" name="Id_Empréstimo"/>
@@ -702,8 +738,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{76E4A97B-7D5A-4E40-82A5-F239AD5B41EF}" name="Pagamentos" displayName="Pagamentos" ref="A1:F2" totalsRowShown="0">
-  <autoFilter ref="A1:F2" xr:uid="{76E4A97B-7D5A-4E40-82A5-F239AD5B41EF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{76E4A97B-7D5A-4E40-82A5-F239AD5B41EF}" name="Pagamentos" displayName="Pagamentos" ref="A1:F3" totalsRowShown="0">
+  <autoFilter ref="A1:F3" xr:uid="{76E4A97B-7D5A-4E40-82A5-F239AD5B41EF}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{198290B1-3A23-491B-9917-F49A606C0044}" name="ID"/>
     <tableColumn id="2" xr3:uid="{8F7769EF-6A96-4E39-BB0F-01679B56A442}" name="Id_parcela"/>
@@ -738,8 +774,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B7C121B-5FD2-43F6-BF02-C8A9170D7250}" name="extrato" displayName="extrato" ref="A1:H3" totalsRowShown="0">
-  <autoFilter ref="A1:H3" xr:uid="{2B7C121B-5FD2-43F6-BF02-C8A9170D7250}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B7C121B-5FD2-43F6-BF02-C8A9170D7250}" name="extrato" displayName="extrato" ref="A1:H9" totalsRowShown="0">
+  <autoFilter ref="A1:H9" xr:uid="{2B7C121B-5FD2-43F6-BF02-C8A9170D7250}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{61AC9B1F-B468-4A3A-BA37-2449BBCCD471}" name="ID"/>
     <tableColumn id="2" xr3:uid="{EE416862-95BC-44B1-9BDB-B15EA35AC103}" name="Categoria"/>
@@ -1071,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAFD19B-6A32-4DA2-B955-DB5C9CCB8233}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
@@ -1148,15 +1184,15 @@
       </c>
       <c r="I2" s="9">
         <f>SUMIFS(extrato[Valor],extrato[ID],participantes[[#This Row],[ID]],extrato[Tipo],"Entrada",extrato[Categoria],"Aplicação")</f>
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="J2" s="9">
-        <f>participantes[[#This Row],[Aplicado]]+(participantes[[#This Row],[Aplicado]]*Geral!C3)</f>
-        <v>30.068787544502584</v>
+        <f ca="1">participantes[[#This Row],[Aplicado]]+(participantes[[#This Row],[Aplicado]]*Geral!C3)</f>
+        <v>2.6397960948443711</v>
       </c>
       <c r="K2" s="9">
-        <f>Geral!$B$3/COUNTA(participantes[ID])</f>
-        <v>30.068787544502584</v>
+        <f ca="1">Geral!$B$3/COUNTA(participantes[ID])</f>
+        <v>2.0531747404345277</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1186,15 +1222,51 @@
       </c>
       <c r="I3" s="9">
         <f>SUMIFS(extrato[Valor],extrato[ID],participantes[[#This Row],[ID]],extrato[Tipo],"Entrada",extrato[Categoria],"Aplicação")</f>
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="J3" s="9">
-        <f>participantes[[#This Row],[Aplicado]]+(participantes[[#This Row],[Aplicado]]*Geral!C3)</f>
-        <v>30.068787544502584</v>
+        <f ca="1">participantes[[#This Row],[Aplicado]]+(participantes[[#This Row],[Aplicado]]*Geral!C3)</f>
+        <v>1.7598640632295854</v>
       </c>
       <c r="K3" s="9">
-        <f>Geral!$B$3/COUNTA(participantes[ID])</f>
-        <v>30.068787544502584</v>
+        <f ca="1">Geral!$B$3/COUNTA(participantes[ID])</f>
+        <v>2.0531747404345277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4">
+        <v>91988468119</v>
+      </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
+      <c r="I4" s="9">
+        <f>SUMIFS(extrato[Valor],extrato[ID],participantes[[#This Row],[ID]],extrato[Tipo],"Entrada",extrato[Categoria],"Aplicação")</f>
+        <v>100</v>
+      </c>
+      <c r="J4" s="9">
+        <f ca="1">participantes[[#This Row],[Aplicado]]+(participantes[[#This Row],[Aplicado]]*Geral!C3)</f>
+        <v>1.7598640632295854</v>
+      </c>
+      <c r="K4" s="9">
+        <f ca="1">Geral!$B$3/COUNTA(participantes[ID])</f>
+        <v>2.0531747404345277</v>
       </c>
     </row>
   </sheetData>
@@ -1205,7 +1277,7 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
     <ignoredError sqref="C2:C3" numberStoredAsText="1"/>
-    <ignoredError sqref="K2:K3 J2:J3" calculatedColumn="1"/>
+    <ignoredError sqref="K2 J2 J3:J4" calculatedColumn="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId3"/>
@@ -1240,7 +1312,7 @@
       </c>
       <c r="B2" s="12">
         <f>SUMIF(extrato[Categoria],"Aplicação",extrato[Valor])</f>
-        <v>100</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1248,12 +1320,12 @@
         <v>36</v>
       </c>
       <c r="B3" s="13">
-        <f>SUMIF(Investimentos[Em posse?],"Sim",Investimentos[Valor real])</f>
-        <v>60.137575089005168</v>
+        <f ca="1">SUMIF(Investimentos[Em posse?],"Sim",Investimentos[Valor real])</f>
+        <v>6.1595242213035837</v>
       </c>
       <c r="C3" s="11">
-        <f>(Tabela5[[#This Row],[Valor]]-B2)*1/B2</f>
-        <v>-0.39862424910994831</v>
+        <f ca="1">(Tabela5[[#This Row],[Valor]]-B2)*1/B2</f>
+        <v>-0.98240135936770412</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1262,7 +1334,7 @@
       </c>
       <c r="B4" s="12">
         <f>SUMIF(extrato[Categoria],"Empréstimo",extrato[Valor])</f>
-        <v>0</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1270,8 +1342,8 @@
         <v>49</v>
       </c>
       <c r="B5" s="13">
-        <f>B3-B4</f>
-        <v>60.137575089005168</v>
+        <f ca="1">B3-B4</f>
+        <v>-443.84047577869643</v>
       </c>
     </row>
   </sheetData>
@@ -1284,11 +1356,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD465C4-726B-4A95-9B15-DA7266B169C4}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.140625" customWidth="1"/>
@@ -1411,40 +1483,235 @@
         <v>20.079999999999998</v>
       </c>
       <c r="F4" s="8">
-        <f>[1]Geral!$C$14/8000</f>
-        <v>2.7490826315158188</v>
+        <v>2.7624766815158188</v>
       </c>
       <c r="G4" s="14">
-        <f>E4*D4</f>
+        <f t="shared" ref="G4:H6" si="0">E4*D4</f>
         <v>30.521599999999999</v>
       </c>
       <c r="H4" s="10">
-        <f>F4*E4</f>
-        <v>55.201579240837638</v>
+        <f t="shared" si="0"/>
+        <v>55.470531764837638</v>
       </c>
       <c r="I4" s="10">
         <f>Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
-        <v>60.137575089005168</v>
+        <v>60.460318117805166</v>
       </c>
       <c r="J4" s="10">
         <f>H4-G4</f>
-        <v>24.679979240837639</v>
+        <v>24.948931764837639</v>
       </c>
       <c r="K4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46030</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2.76</v>
+      </c>
+      <c r="E5" s="8">
+        <v>65.117000000000004</v>
+      </c>
+      <c r="F5" s="8">
+        <v>2.7624766815158188</v>
+      </c>
+      <c r="G5" s="14">
+        <f t="shared" si="0"/>
+        <v>179.72291999999999</v>
+      </c>
+      <c r="H5" s="10">
+        <f t="shared" si="0"/>
+        <v>179.88419407026558</v>
+      </c>
+      <c r="I5" s="10">
+        <f>Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
+        <v>179.9164488843187</v>
+      </c>
+      <c r="J5" s="10">
+        <f>H5-G5</f>
+        <v>0.16127407026559126</v>
+      </c>
+      <c r="K5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="3">
+        <v>46030</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2.76</v>
+      </c>
+      <c r="E6" s="8">
+        <f>85.2-65.06</f>
+        <v>20.14</v>
+      </c>
+      <c r="F6" s="8">
+        <f ca="1">[1]Geral!$C$14/8000</f>
+        <v>2.6650823031606805</v>
+      </c>
+      <c r="G6" s="14">
+        <f t="shared" si="0"/>
+        <v>55.586399999999998</v>
+      </c>
+      <c r="H6" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>53.67475758565611</v>
+      </c>
+      <c r="I6" s="10">
+        <f ca="1">Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
+        <v>53.292429102787331</v>
+      </c>
+      <c r="J6" s="10">
+        <f ca="1">H6-G6</f>
+        <v>-1.9116424143438877</v>
+      </c>
+      <c r="K6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="3">
+        <v>46084</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2.75</v>
+      </c>
+      <c r="E7" s="8">
+        <f>Investimentos[[#This Row],[Total aplicado]]/Investimentos[[#This Row],[Valor Cota]]</f>
+        <v>36.363636363636367</v>
+      </c>
+      <c r="F7" s="8">
+        <f ca="1">[1]Geral!$C$14/8000</f>
+        <v>2.6650823031606805</v>
+      </c>
+      <c r="G7" s="14">
+        <v>100</v>
+      </c>
+      <c r="H7" s="10">
+        <f ca="1">F7*E7</f>
+        <v>96.912083751297487</v>
+      </c>
+      <c r="I7" s="10">
+        <f ca="1">Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
+        <v>96.294500501556982</v>
+      </c>
+      <c r="J7" s="10">
+        <f ca="1">H7-G7</f>
+        <v>-3.0879162487025127</v>
+      </c>
+      <c r="K7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="3">
+        <v>46088</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2.76</v>
+      </c>
+      <c r="E8" s="8">
+        <f>Investimentos[[#This Row],[Total aplicado]]/Investimentos[[#This Row],[Valor Cota]]</f>
+        <v>-15.923913043478263</v>
+      </c>
+      <c r="F8" s="8">
+        <f ca="1">[1]Geral!$C$14/8000</f>
+        <v>2.6650823031606805</v>
+      </c>
+      <c r="G8" s="14">
+        <f>-43.95</f>
+        <v>-43.95</v>
+      </c>
+      <c r="H8" s="10">
+        <f ca="1">F8*E8</f>
+        <v>-42.43853884924345</v>
+      </c>
+      <c r="I8" s="10">
+        <f ca="1">Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
+        <v>-42.136246619092141</v>
+      </c>
+      <c r="J8" s="10">
+        <f ca="1">H8-G8</f>
+        <v>1.5114611507565527</v>
+      </c>
+      <c r="K8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46088</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2.74</v>
+      </c>
+      <c r="E9" s="8">
+        <f>50/D9+E8</f>
+        <v>2.3242621390034852</v>
+      </c>
+      <c r="F9" s="8">
+        <f ca="1">[1]Geral!$C$14/8000</f>
+        <v>2.6650823031606805</v>
+      </c>
+      <c r="G9" s="14">
+        <f>E9*D9</f>
+        <v>6.3684782608695496</v>
+      </c>
+      <c r="H9" s="10">
+        <f ca="1">F9*E9</f>
+        <v>6.1943498945645779</v>
+      </c>
+      <c r="I9" s="10">
+        <f ca="1">Investimentos[[#This Row],[Lucro]]+(Investimentos[[#This Row],[Lucro]]*0.2)+Investimentos[[#This Row],[Total aplicado]]</f>
+        <v>6.1595242213035837</v>
+      </c>
+      <c r="J9" s="10">
+        <f ca="1">H9-G9</f>
+        <v>-0.17412836630497175</v>
+      </c>
+      <c r="K9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E7" s="10"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I10" s="10"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E15" s="8">
+        <f>SUM(E6:E7)</f>
+        <v>56.503636363636367</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="8">
+        <f>E15-E8</f>
+        <v>72.427549407114626</v>
+      </c>
+      <c r="G16" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="E4 E2:K3" calculatedColumn="1"/>
+    <ignoredError sqref="E4 E2:K3 F4:F5 E5:E7 G7" calculatedColumn="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1454,7 +1721,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC02609B-7B27-400D-8043-3B2EE9A1AD1B}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -1463,7 +1730,7 @@
     <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.42578125" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.140625" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
     <col min="11" max="11" width="12.42578125" customWidth="1"/>
@@ -1520,16 +1787,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="3">
-        <v>46052</v>
+        <v>46065</v>
       </c>
       <c r="D2" s="3">
-        <v>46059</v>
+        <v>46093</v>
       </c>
       <c r="E2" s="3">
-        <v>46087</v>
+        <v>46124</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -1538,15 +1805,15 @@
         <v>4.0800000000000003E-2</v>
       </c>
       <c r="H2" s="9">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="I2" s="9">
         <f>Tabela7[[#This Row],[Valor]]+(Tabela7[[#This Row],[Valor]]*(Tabela7[[#This Row],[Juros]]*Tabela7[[#This Row],[Parcelas]]))</f>
-        <v>10.816000000000001</v>
+        <v>129.792</v>
       </c>
       <c r="J2" s="10">
         <f>Tabela7[[#This Row],[Valor final]]/Tabela7[[#This Row],[Parcelas]]</f>
-        <v>5.4080000000000004</v>
+        <v>64.896000000000001</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1556,28 +1823,27 @@
       </c>
       <c r="M2" s="10">
         <f>Tabela7[[#This Row],[Valor final]]-Tabela7[[#This Row],[Valor pago]]</f>
-        <v>10.816000000000001</v>
-      </c>
-      <c r="N2" t="str">
-        <f ca="1">IF(TODAY()&gt;Tabela7[[#This Row],[Próximo Venc.]],"Vencido","À pagar")</f>
-        <v>Vencido</v>
+        <v>129.792</v>
+      </c>
+      <c r="N2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="3">
-        <v>46052</v>
+        <v>46080</v>
       </c>
       <c r="D3" s="3">
-        <v>46087</v>
+        <v>46108</v>
       </c>
       <c r="E3" s="3">
-        <v>46087</v>
+        <v>46139</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -1586,28 +1852,69 @@
         <v>4.0800000000000003E-2</v>
       </c>
       <c r="H3" s="9">
-        <v>10</v>
+        <v>250</v>
       </c>
       <c r="I3" s="9">
         <f>Tabela7[[#This Row],[Valor]]+(Tabela7[[#This Row],[Valor]]*(Tabela7[[#This Row],[Juros]]*Tabela7[[#This Row],[Parcelas]]))</f>
-        <v>10.816000000000001</v>
-      </c>
-      <c r="J3" s="9">
+        <v>270.39999999999998</v>
+      </c>
+      <c r="J3">
         <f>Tabela7[[#This Row],[Valor final]]/Tabela7[[#This Row],[Parcelas]]</f>
-        <v>5.4080000000000004</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="K3">
-        <f ca="1">SUMIF(Tabela7[ID],Tabela7[[#This Row],[ID]],K2)</f>
         <v>0</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
-      <c r="M3" s="9">
-        <f ca="1">Tabela7[[#This Row],[Valor final]]-Tabela7[[#This Row],[Valor pago]]</f>
-        <v>10.816000000000001</v>
+      <c r="M3">
+        <f>Tabela7[[#This Row],[Valor final]]-Tabela7[[#This Row],[Valor pago]]</f>
+        <v>270.39999999999998</v>
       </c>
       <c r="N3" t="str">
+        <f ca="1">IF(TODAY()&gt;Tabela7[[#This Row],[Próximo Venc.]],"Vencido","À pagar")</f>
+        <v>À pagar</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46087</v>
+      </c>
+      <c r="D4" s="3">
+        <v>46118</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46118</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="11">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="H4" s="9">
+        <v>200</v>
+      </c>
+      <c r="I4" s="9">
+        <f>Tabela7[[#This Row],[Valor]]+(Tabela7[[#This Row],[Valor]]*(Tabela7[[#This Row],[Juros]]*Tabela7[[#This Row],[Parcelas]]))</f>
+        <v>208.16</v>
+      </c>
+      <c r="J4">
+        <f>Tabela7[[#This Row],[Valor final]]/Tabela7[[#This Row],[Parcelas]]</f>
+        <v>208.16</v>
+      </c>
+      <c r="M4">
+        <f>Tabela7[[#This Row],[Valor final]]-Tabela7[[#This Row],[Valor pago]]</f>
+        <v>208.16</v>
+      </c>
+      <c r="N4" t="str">
         <f ca="1">IF(TODAY()&gt;Tabela7[[#This Row],[Próximo Venc.]],"Vencido","À pagar")</f>
         <v>À pagar</v>
       </c>
@@ -1622,7 +1929,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ADA09BE-9531-4266-82AC-DE548FACC94B}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -1635,6 +1942,7 @@
     <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1697,16 +2005,92 @@
       </c>
       <c r="H2">
         <f>Emprestimos[[#This Row],[Valor final]]-SUMIF(Pagamentos[ID_empréstimo],Emprestimos[[#This Row],[ID]],Pagamentos[Valor pago])</f>
-        <v>129.792</v>
+        <v>-8.0000000000097771E-3</v>
       </c>
       <c r="I2">
         <f>COUNTIFS(Parcelas[[#All],[Status]],"Em aberto",Parcelas[[#All],[Id_Empréstimo]],Emprestimos[[#This Row],[ID]])</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
         <v>46124</v>
       </c>
       <c r="K2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46080</v>
+      </c>
+      <c r="D3">
+        <v>250</v>
+      </c>
+      <c r="E3" s="11">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <f>Emprestimos[[#This Row],[Valor]]+(Emprestimos[[#This Row],[Valor]]*(Emprestimos[[#This Row],[Juros]]*Emprestimos[[#This Row],[Parcelas]]))-H2</f>
+        <v>270.40800000000002</v>
+      </c>
+      <c r="H3">
+        <f>Emprestimos[[#This Row],[Valor final]]-SUMIF(Pagamentos[ID_empréstimo],Emprestimos[[#This Row],[ID]],Pagamentos[Valor pago])</f>
+        <v>270.40800000000002</v>
+      </c>
+      <c r="I3">
+        <f>COUNTIFS(Parcelas[[#All],[Status]],"Em aberto",Parcelas[[#All],[Id_Empréstimo]],Emprestimos[[#This Row],[ID]])</f>
+        <v>2</v>
+      </c>
+      <c r="J3" s="3">
+        <v>46139</v>
+      </c>
+      <c r="K3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46088</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+      <c r="E4" s="11">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <f>Emprestimos[[#This Row],[Valor]]+(Emprestimos[[#This Row],[Valor]]*(Emprestimos[[#This Row],[Juros]]*Emprestimos[[#This Row],[Parcelas]]))</f>
+        <v>208.16</v>
+      </c>
+      <c r="H4">
+        <f>Emprestimos[[#This Row],[Valor final]]-SUMIF(Pagamentos[ID_empréstimo],Emprestimos[[#This Row],[ID]],Pagamentos[Valor pago])</f>
+        <v>208.16</v>
+      </c>
+      <c r="I4">
+        <f>COUNTIFS(Parcelas[[#All],[Status]],"Em aberto",Parcelas[[#All],[Id_Empréstimo]],Emprestimos[[#This Row],[ID]])</f>
+        <v>1</v>
+      </c>
+      <c r="J4" s="3">
+        <v>46088</v>
+      </c>
+      <c r="K4" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1720,13 +2104,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA33D6C7-F630-4A1D-83C2-01D1A4DFA421}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1773,7 +2157,7 @@
       </c>
       <c r="G2" t="str">
         <f>IF(COUNTIF(Pagamentos[Id_parcela],Parcelas[[#This Row],[ID]])&gt;0,"Pago","Em aberto")</f>
-        <v>Em aberto</v>
+        <v>Pago</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1795,6 +2179,75 @@
         <v>64.896000000000001</v>
       </c>
       <c r="G3" t="str">
+        <f>IF(COUNTIF(Pagamentos[Id_parcela],Parcelas[[#This Row],[ID]])&gt;0,"Pago","Em aberto")</f>
+        <v>Pago</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
+        <f>DATE(YEAR(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)),MONTH(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + Parcelas[[#This Row],[Parcela]], DAY(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + 5)</f>
+        <v>46113</v>
+      </c>
+      <c r="E4" s="9">
+        <f>VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],7,0)/VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],6,0)</f>
+        <v>135.20400000000001</v>
+      </c>
+      <c r="G4" t="str">
+        <f>IF(COUNTIF(Pagamentos[Id_parcela],Parcelas[[#This Row],[ID]])&gt;0,"Pago","Em aberto")</f>
+        <v>Em aberto</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3">
+        <f>DATE(YEAR(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)),MONTH(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + Parcelas[[#This Row],[Parcela]], DAY(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + 5)</f>
+        <v>46144</v>
+      </c>
+      <c r="E5" s="9">
+        <f>VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],7,0)/VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],6,0)</f>
+        <v>135.20400000000001</v>
+      </c>
+      <c r="G5" t="str">
+        <f>IF(COUNTIF(Pagamentos[Id_parcela],Parcelas[[#This Row],[ID]])&gt;0,"Pago","Em aberto")</f>
+        <v>Em aberto</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3">
+        <f>DATE(YEAR(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)),MONTH(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + Parcelas[[#This Row],[Parcela]], DAY(VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],3,0)) + 5)</f>
+        <v>46124</v>
+      </c>
+      <c r="E6" s="9">
+        <f>VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],7,0)/VLOOKUP(Parcelas[[#This Row],[Id_Empréstimo]],Emprestimos[],6,0)</f>
+        <v>208.16</v>
+      </c>
+      <c r="G6" t="str">
         <f>IF(COUNTIF(Pagamentos[Id_parcela],Parcelas[[#This Row],[ID]])&gt;0,"Pago","Em aberto")</f>
         <v>Em aberto</v>
       </c>
@@ -1812,7 +2265,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922C499B-3A06-4A65-996F-FA55853D1BAC}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.28515625" customWidth="1"/>
@@ -1847,19 +2300,43 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" t="e">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <f>VLOOKUP(Pagamentos[[#This Row],[Id_parcela]],Parcelas[],2,0)</f>
-        <v>#N/A</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3">
-        <v>46054</v>
-      </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10" t="e">
+        <v>46079</v>
+      </c>
+      <c r="E2" s="9">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="F2" s="10">
         <f>IFERROR(F1-E2,VLOOKUP(Pagamentos[[#This Row],[ID_empréstimo]],Emprestimos[],7,0)-Pagamentos[[#This Row],[Valor pago]])</f>
-        <v>#N/A</v>
+        <v>64.891999999999996</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <f>VLOOKUP(Pagamentos[[#This Row],[Id_parcela]],Parcelas[],2,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46079</v>
+      </c>
+      <c r="E3" s="9">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="F3">
+        <f>IFERROR(F2-E3,VLOOKUP(Pagamentos[[#This Row],[ID_empréstimo]],Emprestimos[],7,0)-Pagamentos[[#This Row],[Valor pago]])</f>
+        <v>-8.0000000000097771E-3</v>
       </c>
     </row>
   </sheetData>
@@ -1883,7 +2360,7 @@
     <col min="3" max="3" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1973,7 +2450,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FC0C162-5762-4C8E-B0A5-558ECDA215A4}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.85546875" customWidth="1"/>
@@ -2061,6 +2538,156 @@
         <v>85</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="4">
+        <v>50</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46079</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="4">
+        <v>50</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46080</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="4">
+        <v>250</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46080</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="4">
+        <v>100</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46084</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="4">
+        <v>200</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46087</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="4">
+        <v>50</v>
+      </c>
+      <c r="E9" s="3">
+        <v>46088</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H9" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">

</xml_diff>